<commit_message>
AI plan builder kit, plans sized to you, and adherence features
- AI Plan Builder: brief + food list for any AI, 'Paste from AI' import,
  per-day framework report, copyable fix-list, check-plan CLI
- Plans sized to the person's calories, micros first (no completed tile is
  ever lost when sizing down); dislikes auto-swapped by closest micro match
- Prep day, household-aware grocery list with pantry, cook mode with timers,
  local reminders (meal times, night-before prep, evening check)
- 'Life happened' rescue, weekly check-in, 30-day report card, supplements
- Apple Health / Health Connect nutrition export (needs a device build)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MTjfgC7bXJ5Zk8VKro3ypd
</commit_message>
<xml_diff>
--- a/templates/MealPlan_Template.xlsx
+++ b/templates/MealPlan_Template.xlsx
@@ -8,14 +8,16 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingredients" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foods" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SwapGroups" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Brief" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meals" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingredients" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foods" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SwapGroups" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Foods'!$A$1:$C$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Foods'!$A$1:$C$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +125,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -803,6 +817,1070 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t># Eighty: meal plan builder brief</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Paste this whole document into an AI chat, attach **AI_Food_List.csv**, then ask for a plan. For example: *"Write a 7-day Mediterranean plan, 1800–2000 kcal, pescatarian."*</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>## Your role</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>You are writing a meal plan for **Eighty**, an app whose meal plans are built to cover a person's vitamins and minerals every day. People follow the plan meal by meal, and the app tracks every nutrient from the exact foods and grams you choose. Your plan must be **real food people would actually cook**, and it must **pass the nutrition rules below**.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>## Hard rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>1. **Use only foods from AI_Food_List.csv.** Put the exact `food_id` in every ingredient row. Never invent a food_id. If a food you want isn't on the list, pick the closest one that is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>2. **Grams are for the food as listed.** If the food is "Lentils, boiled", the grams are for boiled lentils, not dry ones. Use realistic portions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>3. **Never write nutrition numbers.** The app calculates everything from food_id and grams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>4. **Every day must land inside the plan's calorie band** (calorie_min to calorie_max).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>5. **Each day has a breakfast, a lunch and a dinner**, plus 0–2 snacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>## Nutrition targets (every day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>The app checks every day against an adult man and an adult woman (31–50), so the targets below are the stricter of the two. A nutrient passes at **80%** of the reference amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>| Nutrient | Pass at (per day) | Good sources to reach for |</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>|---|---|---|</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin A | 720 µg RAE | sweet potato, carrots, spinach, kale |</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin C | 72 mg | kiwi, red bell pepper, strawberries, orange, broccoli |</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin D | 12 µg | salmon, sardines, mackerel, trout, eggs *(hard; do your best)* |</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin E | 12 mg | almonds, sunflower seeds, spinach, avocado, olive oil |</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin K | 96 µg | kale, spinach, broccoli, Brussels sprouts |</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>| Thiamin (B1) | 0.96 mg | pork tenderloin, legumes, oats, sunflower seeds |</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>| Riboflavin (B2) | 1.04 mg | dairy, eggs, almonds, mushrooms |</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>| Niacin (B3) | 12.8 mg | chicken, tuna, salmon, peanuts |</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>| Pantothenic acid (B5) | 4 mg | mushrooms, avocado, eggs, sunflower seeds |</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin B6 | 1.04 mg | chickpeas, salmon, chicken, potato, banana |</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>| Folate | 320 µg DFE | lentils, chickpeas, black beans, spinach, asparagus |</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>| Vitamin B12 | 1.92 µg | fish, eggs, dairy, meat *(vegan: fortified nutritional yeast or soy milk)* |</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>| Choline | 440 mg | eggs, fish, chicken, soy *(often the hardest; eggs help most)* |</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>| Calcium | 800 mg | Greek yogurt, milk, cheese, tofu (calcium-set), sardines, kale |</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>| Iron | 14.4 mg | lentils, chickpeas, spinach, pumpkin seeds, beef *(pair plant iron with vitamin C)* |</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>| Magnesium | 336 mg | pumpkin seeds, almonds, black beans, spinach, quinoa |</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>| Phosphorus | 560 mg | dairy, fish, legumes, seeds |</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>| Potassium | 2,720 mg | potatoes, beans, lentils, spinach, banana, yogurt |</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>| Zinc | 8.8 mg | beef, pumpkin seeds, chickpeas, oats, yogurt |</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>| Copper | 0.72 mg | cashews, sunflower seeds, lentils, dark chocolate |</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>| Manganese | 1.84 mg | oats, brown rice, quinoa, nuts, legumes |</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>| Selenium | 44 µg | Brazil nuts (1 nut is plenty), tuna, sardines, eggs |</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>| Iodine | 120 µg | cod, yogurt, milk, eggs, seaweed *(hard; do your best)* |</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>| Fiber | 30 g | legumes, vegetables, berries, oats, chia |</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>### Framework rules (every day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>- **Saturated fat ≤ 10% of calories.** Favour olive oil, fish, legumes and lean poultry over butter, cheese, coconut and fatty meat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>- **Omega-6 : omega-3 ratio ≤ 4 : 1.** Include fatty fish, chia, ground flax or walnuts; avoid seed-oil-heavy cooking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>- **Low glycemic load (≤ 100 per day).** Base carbs on legumes, quinoa, oats, barley and other whole grains, not white rice, white bread or pasta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>- **Protein ≥ 20% of calories**, spread across the day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>- **Fatty fish at least 2 times per 7 days** (salmon, sardines, mackerel, trout, herring), unless the plan is vegetarian or vegan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>- Whole, minimally processed foods. No sweets as snacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>## Swap groups (optional, but please use them)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>When an ingredient could be swapped for something similar, put its group key in `swap_group`. The app then lets people swap it and recalculates. Use only these keys:</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>`leafy_greens`, `legumes`, `low_gi_grains`, `vit_c_fruit`, `berries`, `fatty_fish`, `lean_protein`, `nuts_seeds`, `dairy_protein`, `healthy_oils`</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>## Output format: exactly three CSV blocks, nothing else in between</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
+        <is>
+          <t>```</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>=== PLANS ===</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>plan_id,plan_name,calorie_min,calorie_max,cuisine,tags,description,author,version</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>=== MEALS ===</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>plan_id,day,slot,meal_id,meal_name,prep_minutes,instructions,photo_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>=== INGREDIENTS ===</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>meal_id,food_id,food_name,grams,swap_group,note</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>```</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>Column rules:</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
+        <is>
+          <t>- `plan_id`: short, lowercase, hyphenated, unique (`med-reset-7`). Same id in PLANS and MEALS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>- `tags`: separate several with `|` (e.g. `pescatarian|high-fiber`). Use from: vegetarian, vegan, pescatarian, dairy-free, gluten-free, high-protein, high-fiber.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
+        <is>
+          <t>- `cuisine`: Mediterranean, North American, Asian fusion, Middle Eastern, Mexican, Indian, Japanese, Italian, Caribbean, West African, or Other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>- `day`: 1, 2, 3…</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
+        <is>
+          <t>- `slot`: breakfast, lunch, dinner or snack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
+        <is>
+          <t>- `meal_id`: unique across the plan, e.g. `med7-d1-breakfast`, `med7-d1-snack-2`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>- `instructions`: 1–3 plain sentences. Put commas inside double quotes, e.g. `"Toss the greens, chickpeas and oil."`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
+        <is>
+          <t>- `photo_url`: leave empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>- `food_name`: copy the name from the food list (helps a human read it). `food_id` is what counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
+        <is>
+          <t>- `grams`: a number, no units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>- `note`: optional prep note ("drained", "chopped").</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
+        <is>
+          <t>- `version`: 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>## Before you answer, check yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>For each day, tally calories from the food list and confirm the total is inside the band. Then check the nutrients that most often fall short: **vitamin E, choline, calcium, iron, magnesium, potassium, vitamin D, folate**. If one is short, add or enlarge a food from the table above. Then confirm saturated fat, fish and carb choices against the framework rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>## Fixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="inlineStr">
+        <is>
+          <t>The owner will upload your plan to the app. If anything fails, they'll paste back a **fix list** (e.g. "Day 2: Vitamin E at 61%… Fix: add or increase one of: almonds-raw, sunflower-seeds…"). Apply every fix and return **all three blocks in full** again, not just the changed rows.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Nutrient</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Pass at (per day)</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Good sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin A</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="n">
+        <v>720</v>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>µg RAE</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>sweet potato, carrots, spinach, kale</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin C</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>kiwi, red bell pepper, strawberries, orange, broccoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin D</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>µg</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>salmon, sardines, mackerel, trout, eggs *(hard; do your best)*</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin E</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>almonds, sunflower seeds, spinach, avocado, olive oil</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin K</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>96</v>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>µg</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>kale, spinach, broccoli, Brussels sprouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Thiamin (B1)</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>pork tenderloin, legumes, oats, sunflower seeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Riboflavin (B2)</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>dairy, eggs, almonds, mushrooms</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Niacin (B3)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>chicken, tuna, salmon, peanuts</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Pantothenic acid (B5)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>mushrooms, avocado, eggs, sunflower seeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin B6</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>chickpeas, salmon, chicken, potato, banana</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Folate</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>µg DFE</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>lentils, chickpeas, black beans, spinach, asparagus</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Vitamin B12</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>µg</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>fish, eggs, dairy, meat *(vegan: fortified nutritional yeast or soy milk)*</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Choline</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>440</v>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>eggs, fish, chicken, soy *(often the hardest; eggs help most)*</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Calcium</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>800</v>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Greek yogurt, milk, cheese, tofu (calcium-set), sardines, kale</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>lentils, chickpeas, spinach, pumpkin seeds, beef *(pair plant iron with vitamin C)*</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Magnesium</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>336</v>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>pumpkin seeds, almonds, black beans, spinach, quinoa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Phosphorus</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="n">
+        <v>560</v>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>dairy, fish, legumes, seeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Potassium</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>2720</v>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>potatoes, beans, lentils, spinach, banana, yogurt</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Zinc</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>beef, pumpkin seeds, chickpeas, oats, yogurt</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>cashews, sunflower seeds, lentils, dark chocolate</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Manganese</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>oats, brown rice, quinoa, nuts, legumes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Selenium</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>µg</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Brazil nuts (1 nut is plenty), tuna, sardines, eggs</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Iodine</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>120</v>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>µg</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>cod, yogurt, milk, eggs, seaweed *(hard; do your best)*</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Fiber</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>legumes, vegetables, berries, oats, chia</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F6F54"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -930,7 +2008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F6F54"/>
@@ -1043,7 +2121,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F6F54"/>
@@ -1132,7 +2210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00999999"/>
@@ -3347,7 +4425,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00999999"/>

</xml_diff>